<commit_message>
Fix critical errors by device report
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/es.xlsx
+++ b/api/templates/critical_errors_by_device/es.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="69">
   <si>
     <t xml:space="preserve">Errores por dispositivos</t>
   </si>
@@ -93,49 +93,43 @@
     <t xml:space="preserve">Other Error</t>
   </si>
   <si>
-    <t xml:space="preserve">No Results</t>
-  </si>
-  <si>
     <t xml:space="preserve">Invalid Results</t>
   </si>
   <si>
     <t xml:space="preserve">Total errors, invalid results, no results</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;error_5011&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_5007&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_5006&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_2008&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_2005&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_2037&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_2025&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_2022&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;error_other&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;mtbNoResult&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;mtbInvalid&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;total&gt;</t>
+    <t xml:space="preserve">&lt;deviceName&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;5011&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;5007&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;5006&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;2008&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;2005&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;2037&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;2025&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;2022&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;otherErrors&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;invalidResults&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Code</t>
@@ -241,11 +235,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
-    <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -315,7 +308,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -337,27 +330,6 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -384,7 +356,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -457,19 +429,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -559,13 +523,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="11.0703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.11328125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="15"/>
   </cols>
   <sheetData>
@@ -678,10 +642,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultColWidth="9.6640625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr defaultColWidth="9.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -748,16 +713,13 @@
       <c r="K9" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="17" t="s">
         <v>24</v>
-      </c>
-      <c r="M9" s="17" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>26</v>
@@ -789,11 +751,9 @@
       <c r="K10" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="L10" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M10" s="21" t="s">
-        <v>37</v>
+      <c r="L10" s="19" t="e">
+        <f aca="false">B10+C10+D10+E10+F10+G10+H10+I10+J10+K10</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -813,7 +773,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="9.6640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.69921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.97"/>
@@ -821,300 +781,300 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="22" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="21" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="n">
-        <v>1001</v>
-      </c>
-      <c r="B2" s="23" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="23" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="n">
-        <v>1002</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="23" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="n">
-        <v>1004</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="23" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
-        <v>1005</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="23" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="n">
-        <v>1006</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="23" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="21" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="n">
-        <v>1007</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="23" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="21" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
-        <v>1017</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="23" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="n">
-        <v>1018</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="23" t="s">
+      <c r="C10" s="21" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B10" s="23" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="23" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="21" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="23" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="23" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
-        <v>2009</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="23" t="s">
+      <c r="C14" s="21" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B14" s="23" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="23" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="23" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="23" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B17" s="23" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="n">
+        <v>2037</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="n">
+        <v>4010</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="n">
+        <v>4017</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="23" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="n">
-        <v>2032</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="n">
-        <v>2034</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="n">
-        <v>2037</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="n">
-        <v>4010</v>
-      </c>
-      <c r="B23" s="23" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="n">
+        <v>5006</v>
+      </c>
+      <c r="B25" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C25" s="21" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="n">
-        <v>4017</v>
-      </c>
-      <c r="B24" s="23" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="n">
+        <v>5007</v>
+      </c>
+      <c r="B26" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="23" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="n">
-        <v>5006</v>
-      </c>
-      <c r="B25" s="23" t="s">
+      <c r="C26" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="23" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="n">
+        <v>5011</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="n">
-        <v>5007</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="n">
-        <v>5011</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>